<commit_message>
Add depth model and update form on measurements
</commit_message>
<xml_diff>
--- a/static/download_template/monitoring_data.xlsx
+++ b/static/download_template/monitoring_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Groundwater Level" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Groundwater Quality" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Abstraction-Discharge" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Groundwater Level" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Groundwater Quality" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Abstraction-Discharge" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="22">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -40,6 +40,12 @@
   </si>
   <si>
     <t xml:space="preserve">Unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depth Unit</t>
   </si>
   <si>
     <t xml:space="preserve">Methodology</t>
@@ -66,6 +72,9 @@
     <t xml:space="preserve">Unit must be either: 
 • m 
 • ft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The numeric value of the depth of measurement.</t>
   </si>
   <si>
     <t xml:space="preserve">Explain the methodology used to collect the data, in the field and eventually in the lab.</t>
@@ -318,32 +327,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -419,69 +432,187 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF953735"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMJ2"/>
+  <dimension ref="A1:AML2"/>
   <sheetFormatPr defaultColWidth="15.71484375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="26.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35.7"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="5" style="1" width="15.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="9.14"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="5" style="1" width="15.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1026" min="1026" style="2" width="9.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" s="5" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AMJ1" s="0"/>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="AML1" s="2"/>
     </row>
-    <row r="2" s="6" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="5" t="s">
+    <row r="2" s="7" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="AMJ2" s="0"/>
+      <c r="F2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="AML2" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -495,68 +626,80 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF953735"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMJ2"/>
+  <dimension ref="A1:AML2"/>
   <sheetFormatPr defaultColWidth="15.71484375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="26.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35.7"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="5" style="1" width="15.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="9.14"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="5" style="1" width="15.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1026" min="1026" style="2" width="9.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" s="5" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AMJ1" s="0"/>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="AML1" s="2"/>
     </row>
-    <row r="2" s="6" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="5" t="s">
+    <row r="2" s="7" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="AMJ2" s="0"/>
+      <c r="AML2" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -570,68 +713,80 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF953735"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMJ2"/>
+  <dimension ref="A1:AML2"/>
   <sheetFormatPr defaultColWidth="15.71484375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="26.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35.7"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="5" style="1" width="15.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="9.14"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="5" style="1" width="15.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1026" min="1026" style="2" width="9.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" s="5" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AMJ1" s="0"/>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="AML1" s="2"/>
     </row>
-    <row r="2" s="6" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="5" t="s">
+    <row r="2" s="7" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="AMJ2" s="0"/>
+      <c r="I2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="AML2" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Depth measurement feature (#229)
* Add depth model and update form on measurements

* Fix tests

* Clean print
</commit_message>
<xml_diff>
--- a/static/download_template/monitoring_data.xlsx
+++ b/static/download_template/monitoring_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Groundwater Level" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Groundwater Quality" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Abstraction-Discharge" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Groundwater Level" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Groundwater Quality" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Abstraction-Discharge" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="22">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -40,6 +40,12 @@
   </si>
   <si>
     <t xml:space="preserve">Unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depth Unit</t>
   </si>
   <si>
     <t xml:space="preserve">Methodology</t>
@@ -66,6 +72,9 @@
     <t xml:space="preserve">Unit must be either: 
 • m 
 • ft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The numeric value of the depth of measurement.</t>
   </si>
   <si>
     <t xml:space="preserve">Explain the methodology used to collect the data, in the field and eventually in the lab.</t>
@@ -318,32 +327,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -419,69 +432,187 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF953735"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMJ2"/>
+  <dimension ref="A1:AML2"/>
   <sheetFormatPr defaultColWidth="15.71484375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="26.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35.7"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="5" style="1" width="15.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="9.14"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="5" style="1" width="15.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1026" min="1026" style="2" width="9.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" s="5" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AMJ1" s="0"/>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="AML1" s="2"/>
     </row>
-    <row r="2" s="6" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="5" t="s">
+    <row r="2" s="7" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="AMJ2" s="0"/>
+      <c r="F2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="AML2" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -495,68 +626,80 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF953735"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMJ2"/>
+  <dimension ref="A1:AML2"/>
   <sheetFormatPr defaultColWidth="15.71484375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="26.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35.7"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="5" style="1" width="15.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="9.14"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="5" style="1" width="15.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1026" min="1026" style="2" width="9.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" s="5" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AMJ1" s="0"/>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="AML1" s="2"/>
     </row>
-    <row r="2" s="6" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="5" t="s">
+    <row r="2" s="7" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="AMJ2" s="0"/>
+      <c r="AML2" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -570,68 +713,80 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <tabColor rgb="FF953735"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMJ2"/>
+  <dimension ref="A1:AML2"/>
   <sheetFormatPr defaultColWidth="15.71484375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="26.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35.7"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1023" min="5" style="1" width="15.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="9.14"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1025" min="5" style="1" width="15.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1026" min="1026" style="2" width="9.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" s="5" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AMJ1" s="0"/>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="AML1" s="2"/>
     </row>
-    <row r="2" s="6" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="5" t="s">
+    <row r="2" s="7" customFormat="true" ht="159.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="AMJ2" s="0"/>
+      <c r="I2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="AML2" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>